<commit_message>
fix: change trigger name to be company name
</commit_message>
<xml_diff>
--- a/보유계약실행일자.xlsx
+++ b/보유계약실행일자.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\QuintetCompany\projects\insurance_auto_login_ms_uipath\UI_Path_Project\Test_Create_Time_Trigger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92F04205-6E99-42A4-976E-580E021C7079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C9E9E6-98FE-483D-B57D-A1A4D0747643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,6 @@
     <t>19, 20, 21</t>
   </si>
   <si>
-    <t>22, 23, 24</t>
-  </si>
-  <si>
     <t>08:30</t>
   </si>
   <si>
@@ -100,7 +97,10 @@
     <t>22:30</t>
   </si>
   <si>
-    <t>1, 2, 3, 4</t>
+    <t>1, 2, 3, 4, 5, 6, 7, 8, 9, 10</t>
+  </si>
+  <si>
+    <t>21, 22, 23, 24, 25</t>
   </si>
 </sst>
 </file>
@@ -504,7 +504,7 @@
         <v>26</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -515,7 +515,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -526,7 +526,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -537,7 +537,7 @@
         <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -548,7 +548,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -559,7 +559,7 @@
         <v>15</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -570,7 +570,7 @@
         <v>16</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -578,10 +578,10 @@
         <v>10</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>